<commit_message>
Update tuned model — Macro F1 improved from 91.74% to 96.87%
</commit_message>
<xml_diff>
--- a/tables/classification_report.xlsx
+++ b/tables/classification_report.xlsx
@@ -465,10 +465,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9986666666666667</v>
+        <v>0.9996666666666667</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9993328885923949</v>
+        <v>0.9998333055509252</v>
       </c>
       <c r="E2" t="n">
         <v>6000</v>
@@ -481,13 +481,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9624177346726706</v>
+        <v>0.9871086556169429</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9261666666666667</v>
+        <v>0.9826666666666667</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9439442840156277</v>
+        <v>0.9848826526350957</v>
       </c>
       <c r="E3" t="n">
         <v>6000</v>
@@ -500,13 +500,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.998970310622962</v>
+        <v>0.991930060524546</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9701666666666666</v>
+        <v>0.9833333333333333</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9843578253149573</v>
+        <v>0.987612989621694</v>
       </c>
       <c r="E4" t="n">
         <v>6000</v>
@@ -519,13 +519,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9418411432369558</v>
+        <v>0.9753231492361927</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9449816605535178</v>
+        <v>0.9686562187395799</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9434087882822902</v>
+        <v>0.971978251777499</v>
       </c>
       <c r="E5" t="n">
         <v>5998</v>
@@ -538,13 +538,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.246353322528363</v>
+        <v>0.7346368715083799</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9712460063897763</v>
+        <v>0.8402555910543131</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3930187459599224</v>
+        <v>0.7839046199701938</v>
       </c>
       <c r="E6" t="n">
         <v>313</v>
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9930321255684319</v>
+        <v>0.9981074392196826</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9855146309506478</v>
+        <v>0.9981074392196826</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9892590968873302</v>
+        <v>0.9981074392196826</v>
       </c>
       <c r="E7" t="n">
         <v>13738</v>
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9952710690761696</v>
+        <v>0.9956529008527002</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9821666666666666</v>
+        <v>0.9925</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9886754466907138</v>
+        <v>0.9940739504215007</v>
       </c>
       <c r="E8" t="n">
         <v>6000</v>
@@ -595,13 +595,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9941520467836257</v>
+        <v>0.9995478182229256</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9997738068310337</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9969550016916657</v>
+        <v>0.9997738579828132</v>
       </c>
       <c r="E9" t="n">
         <v>4421</v>
@@ -614,13 +614,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.9917743830787309</v>
+        <v>0.9878858280783273</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9846666666666667</v>
+        <v>0.9921666666666666</v>
       </c>
       <c r="D10" t="n">
-        <v>0.988207744417496</v>
+        <v>0.9900216198237153</v>
       </c>
       <c r="E10" t="n">
         <v>6000</v>
@@ -633,13 +633,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.9742368095994354</v>
+        <v>0.9714897824653922</v>
       </c>
       <c r="C11" t="n">
-        <v>0.9201666666666667</v>
+        <v>0.9825</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9464301019970858</v>
+        <v>0.976963871395426</v>
       </c>
       <c r="E11" t="n">
         <v>6000</v>
@@ -652,16 +652,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.9694559285596164</v>
+        <v>0.988969737059699</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9694559285596164</v>
+        <v>0.988969737059699</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9694559285596164</v>
+        <v>0.988969737059699</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9694559285596164</v>
+        <v>0.988969737059699</v>
       </c>
     </row>
     <row r="13">
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.9098048945167345</v>
+        <v>0.964168250572509</v>
       </c>
       <c r="C13" t="n">
-        <v>0.9683516104724976</v>
+        <v>0.973985258234691</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9173589923849483</v>
+        <v>0.9687152558398544</v>
       </c>
       <c r="E13" t="n">
         <v>60470</v>
@@ -690,13 +690,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.9806468521461216</v>
+        <v>0.9891737036463008</v>
       </c>
       <c r="C14" t="n">
-        <v>0.9694559285596164</v>
+        <v>0.988969737059699</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9737927908266789</v>
+        <v>0.9890461098568591</v>
       </c>
       <c r="E14" t="n">
         <v>60470</v>

</xml_diff>